<commit_message>
Add user / AI
</commit_message>
<xml_diff>
--- a/label/Results.xlsx
+++ b/label/Results.xlsx
@@ -414,254 +414,228 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Count</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>Percent</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Open Code</t>
-        </is>
-      </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Count</t>
-        </is>
-      </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Percent</t>
+          <t>Overall - N = 258</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Information Seeking</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>44</v>
-      </c>
-      <c r="C2" s="1" t="n">
-        <v>0.09205020920502092</v>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>Information Seeking</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>Requesting direct answer</t>
-        </is>
-      </c>
-      <c r="G2" t="n">
-        <v>29</v>
-      </c>
-      <c r="H2" s="1" t="n">
-        <v>0.06066945606694561</v>
-      </c>
+      <c r="A2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Understanding</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>61</v>
-      </c>
-      <c r="C3" s="1" t="n">
-        <v>0.1276150627615063</v>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Percent</t>
+        </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Information Seeking</t>
+          <t>Category</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Requesting information</t>
-        </is>
-      </c>
-      <c r="G3" t="n">
-        <v>15</v>
-      </c>
-      <c r="H3" s="1" t="n">
-        <v>0.03138075313807531</v>
+          <t>Open Code</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Percent</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Challenge</t>
+          <t>Information Seeking</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>7</v>
+        <v>44</v>
       </c>
       <c r="C4" s="1" t="n">
-        <v>0.01464435146443515</v>
+        <v>0.1705426356589147</v>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Understanding</t>
+          <t>Information Seeking</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Requesting clarification</t>
+          <t>Requesting direct answer</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>53</v>
+        <v>29</v>
       </c>
       <c r="H4" s="1" t="n">
-        <v>0.1108786610878661</v>
+        <v>0.1124031007751938</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Verification</t>
+          <t>Understanding</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>50</v>
+        <v>61</v>
       </c>
       <c r="C5" s="1" t="n">
-        <v>0.104602510460251</v>
+        <v>0.2364341085271318</v>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Understanding</t>
+          <t>Information Seeking</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Requesting justification</t>
+          <t>Requesting information</t>
         </is>
       </c>
       <c r="G5" t="n">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="H5" s="1" t="n">
-        <v>0.01673640167364017</v>
+        <v>0.05813953488372093</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Reliance / Decision</t>
+          <t>Challenge</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="C6" s="1" t="n">
-        <v>0.0104602510460251</v>
+        <v>0.02713178294573643</v>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Challenge</t>
+          <t>Understanding</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Challenging the agent</t>
+          <t>Requesting clarification</t>
         </is>
       </c>
       <c r="G6" t="n">
-        <v>2</v>
+        <v>53</v>
       </c>
       <c r="H6" s="1" t="n">
-        <v>0.004184100418410041</v>
+        <v>0.2054263565891473</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>Verification</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>55</v>
+      </c>
+      <c r="C7" s="1" t="n">
+        <v>0.2131782945736434</v>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Understanding</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>Requesting justification</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>8</v>
+      </c>
+      <c r="H7" s="1" t="n">
+        <v>0.0310077519379845</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Reliance / Decision</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>5</v>
+      </c>
+      <c r="C8" s="1" t="n">
+        <v>0.01937984496124031</v>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Challenge</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>Challenging the agent</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>2</v>
+      </c>
+      <c r="H8" s="1" t="n">
+        <v>0.007751937984496124</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
           <t>Agent Behavior</t>
         </is>
       </c>
-      <c r="B7" t="n">
-        <v>78</v>
-      </c>
-      <c r="C7" s="1" t="n">
-        <v>0.1631799163179916</v>
-      </c>
-      <c r="E7" t="inlineStr">
+      <c r="B9" t="n">
+        <v>86</v>
+      </c>
+      <c r="C9" s="1" t="n">
+        <v>0.3333333333333333</v>
+      </c>
+      <c r="E9" t="inlineStr">
         <is>
           <t>Challenge</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>Proposing an alternative</t>
         </is>
       </c>
-      <c r="G7" t="n">
+      <c r="G9" t="n">
         <v>5</v>
       </c>
-      <c r="H7" s="1" t="n">
-        <v>0.0104602510460251</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>Verification</t>
-        </is>
-      </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>Requesting re-analysis</t>
-        </is>
-      </c>
-      <c r="G8" t="n">
-        <v>18</v>
-      </c>
-      <c r="H8" s="1" t="n">
-        <v>0.03765690376569038</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Verification</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Requesting result verification</t>
-        </is>
-      </c>
-      <c r="G9" t="n">
-        <v>23</v>
-      </c>
       <c r="H9" s="1" t="n">
-        <v>0.04811715481171548</v>
+        <v>0.01937984496124031</v>
       </c>
     </row>
     <row r="10">
@@ -672,14 +646,14 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Requesting data validation</t>
+          <t>Requesting re-analysis</t>
         </is>
       </c>
       <c r="G10" t="n">
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="H10" s="1" t="n">
-        <v>0.01255230125523013</v>
+        <v>0.06976744186046512</v>
       </c>
     </row>
     <row r="11">
@@ -690,50 +664,50 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Requesting assumption validation</t>
+          <t>Requesting result verification</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>8</v>
+        <v>23</v>
       </c>
       <c r="H11" s="1" t="n">
-        <v>0.01673640167364017</v>
+        <v>0.08914728682170543</v>
       </c>
     </row>
     <row r="12">
       <c r="E12" t="inlineStr">
         <is>
-          <t>Reliance / Decision</t>
+          <t>Verification</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Accepting the answer</t>
+          <t>Requesting data validation</t>
         </is>
       </c>
       <c r="G12" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H12" s="1" t="n">
-        <v>0.0104602510460251</v>
+        <v>0.02325581395348837</v>
       </c>
     </row>
     <row r="13">
       <c r="E13" t="inlineStr">
         <is>
-          <t>Reliance / Decision</t>
+          <t>Verification</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Accepting a flawed answer</t>
+          <t>Requesting assumption validation</t>
         </is>
       </c>
       <c r="G13" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="H13" s="1" t="n">
-        <v>0</v>
+        <v>0.0310077519379845</v>
       </c>
     </row>
     <row r="14">
@@ -744,50 +718,50 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Proceeding without resolving concern</t>
+          <t>Accepting the answer</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="H14" s="1" t="n">
-        <v>0</v>
+        <v>0.01937984496124031</v>
       </c>
     </row>
     <row r="15">
       <c r="E15" t="inlineStr">
         <is>
-          <t>Agent Behavior</t>
+          <t>Reliance / Decision</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Relying on pre-existing analysis</t>
+          <t>Accepting a flawed answer</t>
         </is>
       </c>
       <c r="G15" t="n">
-        <v>25</v>
+        <v>0</v>
       </c>
       <c r="H15" s="1" t="n">
-        <v>0.05230125523012552</v>
+        <v>0</v>
       </c>
     </row>
     <row r="16">
       <c r="E16" t="inlineStr">
         <is>
-          <t>Agent Behavior</t>
+          <t>Reliance / Decision</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Exposing an assumption</t>
+          <t>Proceeding without resolving concern</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="H16" s="1" t="n">
-        <v>0.07949790794979079</v>
+        <v>0</v>
       </c>
     </row>
     <row r="17">
@@ -798,14 +772,14 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Identifying an issue</t>
+          <t>Relying on pre-existing analysis</t>
         </is>
       </c>
       <c r="G17" t="n">
-        <v>16</v>
+        <v>25</v>
       </c>
       <c r="H17" s="1" t="n">
-        <v>0.03347280334728033</v>
+        <v>0.09689922480620156</v>
       </c>
     </row>
     <row r="18">
@@ -816,14 +790,890 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
+          <t>Exposing an assumption</t>
+        </is>
+      </c>
+      <c r="G18" t="n">
+        <v>38</v>
+      </c>
+      <c r="H18" s="1" t="n">
+        <v>0.1472868217054264</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Agent Behavior</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Identifying an issue</t>
+        </is>
+      </c>
+      <c r="G19" t="n">
+        <v>16</v>
+      </c>
+      <c r="H19" s="1" t="n">
+        <v>0.06201550387596899</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Agent Behavior</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
           <t>Correcting the result</t>
         </is>
       </c>
-      <c r="G18" t="n">
+      <c r="G20" t="n">
         <v>7</v>
       </c>
-      <c r="H18" s="1" t="n">
-        <v>0.01464435146443515</v>
+      <c r="H20" s="1" t="n">
+        <v>0.02713178294573643</v>
+      </c>
+    </row>
+    <row r="21"/>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>User (Prompt) - N = 172</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Percent</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>Open Code</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>Percent</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Information Seeking</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>44</v>
+      </c>
+      <c r="C25" s="1" t="n">
+        <v>0.2558139534883721</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Information Seeking</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>Requesting direct answer</t>
+        </is>
+      </c>
+      <c r="G25" t="n">
+        <v>29</v>
+      </c>
+      <c r="H25" s="1" t="n">
+        <v>0.1686046511627907</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Understanding</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>61</v>
+      </c>
+      <c r="C26" s="1" t="n">
+        <v>0.3546511627906977</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Information Seeking</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>Requesting information</t>
+        </is>
+      </c>
+      <c r="G26" t="n">
+        <v>15</v>
+      </c>
+      <c r="H26" s="1" t="n">
+        <v>0.0872093023255814</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Challenge</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>7</v>
+      </c>
+      <c r="C27" s="1" t="n">
+        <v>0.04069767441860465</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Understanding</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Requesting clarification</t>
+        </is>
+      </c>
+      <c r="G27" t="n">
+        <v>53</v>
+      </c>
+      <c r="H27" s="1" t="n">
+        <v>0.3081395348837209</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Verification</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>55</v>
+      </c>
+      <c r="C28" s="1" t="n">
+        <v>0.3197674418604651</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Understanding</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>Requesting justification</t>
+        </is>
+      </c>
+      <c r="G28" t="n">
+        <v>8</v>
+      </c>
+      <c r="H28" s="1" t="n">
+        <v>0.04651162790697674</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Reliance / Decision</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>5</v>
+      </c>
+      <c r="C29" s="1" t="n">
+        <v>0.02906976744186046</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Challenge</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>Challenging the agent</t>
+        </is>
+      </c>
+      <c r="G29" t="n">
+        <v>2</v>
+      </c>
+      <c r="H29" s="1" t="n">
+        <v>0.01162790697674419</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Agent Behavior</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>0</v>
+      </c>
+      <c r="C30" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Challenge</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>Proposing an alternative</t>
+        </is>
+      </c>
+      <c r="G30" t="n">
+        <v>5</v>
+      </c>
+      <c r="H30" s="1" t="n">
+        <v>0.02906976744186046</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Verification</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>Requesting re-analysis</t>
+        </is>
+      </c>
+      <c r="G31" t="n">
+        <v>18</v>
+      </c>
+      <c r="H31" s="1" t="n">
+        <v>0.1046511627906977</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Verification</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Requesting result verification</t>
+        </is>
+      </c>
+      <c r="G32" t="n">
+        <v>23</v>
+      </c>
+      <c r="H32" s="1" t="n">
+        <v>0.1337209302325581</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Verification</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Requesting data validation</t>
+        </is>
+      </c>
+      <c r="G33" t="n">
+        <v>6</v>
+      </c>
+      <c r="H33" s="1" t="n">
+        <v>0.03488372093023256</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>Verification</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Requesting assumption validation</t>
+        </is>
+      </c>
+      <c r="G34" t="n">
+        <v>8</v>
+      </c>
+      <c r="H34" s="1" t="n">
+        <v>0.04651162790697674</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Reliance / Decision</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Accepting the answer</t>
+        </is>
+      </c>
+      <c r="G35" t="n">
+        <v>5</v>
+      </c>
+      <c r="H35" s="1" t="n">
+        <v>0.02906976744186046</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>Reliance / Decision</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Accepting a flawed answer</t>
+        </is>
+      </c>
+      <c r="G36" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>Reliance / Decision</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Proceeding without resolving concern</t>
+        </is>
+      </c>
+      <c r="G37" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>Agent Behavior</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Relying on pre-existing analysis</t>
+        </is>
+      </c>
+      <c r="G38" t="n">
+        <v>0</v>
+      </c>
+      <c r="H38" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>Agent Behavior</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Exposing an assumption</t>
+        </is>
+      </c>
+      <c r="G39" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>Agent Behavior</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Identifying an issue</t>
+        </is>
+      </c>
+      <c r="G40" t="n">
+        <v>0</v>
+      </c>
+      <c r="H40" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Agent Behavior</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Correcting the result</t>
+        </is>
+      </c>
+      <c r="G41" t="n">
+        <v>0</v>
+      </c>
+      <c r="H41" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42"/>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>AI (Response) - N = 86</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Percent</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Open Code</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Count</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Percent</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>Information Seeking</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>0</v>
+      </c>
+      <c r="C46" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>Information Seeking</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Requesting direct answer</t>
+        </is>
+      </c>
+      <c r="G46" t="n">
+        <v>0</v>
+      </c>
+      <c r="H46" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Understanding</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>0</v>
+      </c>
+      <c r="C47" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>Information Seeking</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Requesting information</t>
+        </is>
+      </c>
+      <c r="G47" t="n">
+        <v>0</v>
+      </c>
+      <c r="H47" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Challenge</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>0</v>
+      </c>
+      <c r="C48" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>Understanding</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Requesting clarification</t>
+        </is>
+      </c>
+      <c r="G48" t="n">
+        <v>0</v>
+      </c>
+      <c r="H48" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Verification</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>0</v>
+      </c>
+      <c r="C49" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>Understanding</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Requesting justification</t>
+        </is>
+      </c>
+      <c r="G49" t="n">
+        <v>0</v>
+      </c>
+      <c r="H49" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Reliance / Decision</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>0</v>
+      </c>
+      <c r="C50" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>Challenge</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Challenging the agent</t>
+        </is>
+      </c>
+      <c r="G50" t="n">
+        <v>0</v>
+      </c>
+      <c r="H50" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Agent Behavior</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>86</v>
+      </c>
+      <c r="C51" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>Challenge</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>Proposing an alternative</t>
+        </is>
+      </c>
+      <c r="G51" t="n">
+        <v>0</v>
+      </c>
+      <c r="H51" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>Verification</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>Requesting re-analysis</t>
+        </is>
+      </c>
+      <c r="G52" t="n">
+        <v>0</v>
+      </c>
+      <c r="H52" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>Verification</t>
+        </is>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>Requesting result verification</t>
+        </is>
+      </c>
+      <c r="G53" t="n">
+        <v>0</v>
+      </c>
+      <c r="H53" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>Verification</t>
+        </is>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>Requesting data validation</t>
+        </is>
+      </c>
+      <c r="G54" t="n">
+        <v>0</v>
+      </c>
+      <c r="H54" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>Verification</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Requesting assumption validation</t>
+        </is>
+      </c>
+      <c r="G55" t="n">
+        <v>0</v>
+      </c>
+      <c r="H55" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>Reliance / Decision</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>Accepting the answer</t>
+        </is>
+      </c>
+      <c r="G56" t="n">
+        <v>0</v>
+      </c>
+      <c r="H56" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>Reliance / Decision</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>Accepting a flawed answer</t>
+        </is>
+      </c>
+      <c r="G57" t="n">
+        <v>0</v>
+      </c>
+      <c r="H57" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>Reliance / Decision</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>Proceeding without resolving concern</t>
+        </is>
+      </c>
+      <c r="G58" t="n">
+        <v>0</v>
+      </c>
+      <c r="H58" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>Agent Behavior</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>Relying on pre-existing analysis</t>
+        </is>
+      </c>
+      <c r="G59" t="n">
+        <v>25</v>
+      </c>
+      <c r="H59" s="1" t="n">
+        <v>0.2906976744186047</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>Agent Behavior</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>Exposing an assumption</t>
+        </is>
+      </c>
+      <c r="G60" t="n">
+        <v>38</v>
+      </c>
+      <c r="H60" s="1" t="n">
+        <v>0.4418604651162791</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>Agent Behavior</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>Identifying an issue</t>
+        </is>
+      </c>
+      <c r="G61" t="n">
+        <v>16</v>
+      </c>
+      <c r="H61" s="1" t="n">
+        <v>0.186046511627907</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>Agent Behavior</t>
+        </is>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>Correcting the result</t>
+        </is>
+      </c>
+      <c r="G62" t="n">
+        <v>7</v>
+      </c>
+      <c r="H62" s="1" t="n">
+        <v>0.08139534883720931</v>
       </c>
     </row>
   </sheetData>

</xml_diff>